<commit_message>
renamed typo in dc fix pcb. added some docs incl. test procedure for dc fix pcbs
</commit_message>
<xml_diff>
--- a/docs/IM828XCC_LTC6992HS6-4_dutycyc_to_temperature.xlsx
+++ b/docs/IM828XCC_LTC6992HS6-4_dutycyc_to_temperature.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26130"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GIT\UltraZohm\pcb_design\uz_per_sic_inverter_828xcc\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3923F02C-4F4C-4B1C-8CF8-1A63E185827D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9090A09-0D3C-497D-862F-2B9AA65FD688}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="67080" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="13">
   <si>
     <t>Temperature in °C</t>
   </si>
@@ -62,6 +62,18 @@
   </si>
   <si>
     <t>TEMP</t>
+  </si>
+  <si>
+    <t>temp in °C</t>
+  </si>
+  <si>
+    <t>dutycycle</t>
+  </si>
+  <si>
+    <t>measured hw #1</t>
+  </si>
+  <si>
+    <t>measured hw #2</t>
   </si>
 </sst>
 </file>
@@ -135,36 +147,6 @@
     </mc:Fallback>
   </mc:AlternateContent>
   <c:chart>
-    <c:title>
-      <c:overlay val="0"/>
-      <c:spPr>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:effectLst/>
-      </c:spPr>
-      <c:txPr>
-        <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr>
-            <a:defRPr sz="1400" b="0" i="0" u="none" strike="noStrike" kern="1200" spc="0" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1">
-                  <a:lumMod val="65000"/>
-                  <a:lumOff val="35000"/>
-                </a:schemeClr>
-              </a:solidFill>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:defRPr>
-          </a:pPr>
-          <a:endParaRPr lang="de-DE"/>
-        </a:p>
-      </c:txPr>
-    </c:title>
     <c:autoTitleDeleted val="0"/>
     <c:plotArea>
       <c:layout/>
@@ -291,6 +273,129 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000001-5FE0-4630-B64B-256BD0350C49}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>Tabelle1!$I$9</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>measured hw #1</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent2"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="19050" cap="rnd">
+                <a:solidFill>
+                  <a:schemeClr val="accent2"/>
+                </a:solidFill>
+                <a:prstDash val="sysDot"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="linear"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="1"/>
+            <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-0.11203673554138263"/>
+                  <c:y val="2.2545771412361436E-2"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:numFmt formatCode="General" sourceLinked="0"/>
+              <c:spPr>
+                <a:noFill/>
+                <a:ln>
+                  <a:noFill/>
+                </a:ln>
+                <a:effectLst/>
+              </c:spPr>
+              <c:txPr>
+                <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                <a:lstStyle/>
+                <a:p>
+                  <a:pPr>
+                    <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="65000"/>
+                          <a:lumOff val="35000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:latin typeface="+mn-lt"/>
+                      <a:ea typeface="+mn-ea"/>
+                      <a:cs typeface="+mn-cs"/>
+                    </a:defRPr>
+                  </a:pPr>
+                  <a:endParaRPr lang="de-DE"/>
+                </a:p>
+              </c:txPr>
+            </c:trendlineLbl>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Tabelle1!$H$23:$H$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>0.7</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.94</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Tabelle1!$I$23:$I$28</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="6"/>
+                <c:pt idx="0">
+                  <c:v>35</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>26</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000001-5444-481F-AE11-EFE352F6AC0A}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1475,24 +1580,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:J29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="54.08984375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="33.36328125" bestFit="1" customWidth="1"/>
+    <col min="9" max="10" width="14.6328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>1</v>
       </c>
@@ -1503,7 +1609,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B6" t="s">
         <v>7</v>
       </c>
@@ -1514,7 +1620,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -1529,37 +1635,250 @@
         <v>25</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B8" s="2">
         <v>0.15</v>
       </c>
       <c r="C8" s="1">
-        <f t="shared" ref="C8:C13" si="0">B8</f>
+        <f t="shared" ref="C8" si="0">B8</f>
         <v>0.15</v>
       </c>
       <c r="D8">
         <v>125</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B9" s="2"/>
       <c r="C9" s="1"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="I9" t="s">
+        <v>11</v>
+      </c>
+      <c r="J9" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B10" s="2"/>
       <c r="C10" s="1"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E10" t="s">
+        <v>10</v>
+      </c>
+      <c r="F10" t="s">
+        <v>9</v>
+      </c>
+      <c r="H10" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B11" s="2"/>
       <c r="C11" s="1"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E11">
+        <v>0.1</v>
+      </c>
+      <c r="F11">
+        <f>E11*-142.86+146.43</f>
+        <v>132.14400000000001</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B12" s="2"/>
       <c r="C12" s="1"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="E12">
+        <f>E11+0.05</f>
+        <v>0.15000000000000002</v>
+      </c>
+      <c r="F12">
+        <f t="shared" ref="F12:F29" si="1">E12*-142.86+146.43</f>
+        <v>125.001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="B13" s="2"/>
       <c r="C13" s="1"/>
+      <c r="E13">
+        <f t="shared" ref="E13:E29" si="2">E12+0.05</f>
+        <v>0.2</v>
+      </c>
+      <c r="F13">
+        <f t="shared" si="1"/>
+        <v>117.858</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E14">
+        <f t="shared" si="2"/>
+        <v>0.25</v>
+      </c>
+      <c r="F14">
+        <f t="shared" si="1"/>
+        <v>110.715</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E15">
+        <f t="shared" si="2"/>
+        <v>0.3</v>
+      </c>
+      <c r="F15">
+        <f t="shared" si="1"/>
+        <v>103.572</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="E16">
+        <f t="shared" si="2"/>
+        <v>0.35</v>
+      </c>
+      <c r="F16">
+        <f t="shared" si="1"/>
+        <v>96.429000000000002</v>
+      </c>
+    </row>
+    <row r="17" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E17">
+        <f t="shared" si="2"/>
+        <v>0.39999999999999997</v>
+      </c>
+      <c r="F17">
+        <f t="shared" si="1"/>
+        <v>89.286000000000001</v>
+      </c>
+    </row>
+    <row r="18" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E18">
+        <f t="shared" si="2"/>
+        <v>0.44999999999999996</v>
+      </c>
+      <c r="F18">
+        <f t="shared" si="1"/>
+        <v>82.143000000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E19">
+        <f t="shared" si="2"/>
+        <v>0.49999999999999994</v>
+      </c>
+      <c r="F19">
+        <f t="shared" si="1"/>
+        <v>75.000000000000014</v>
+      </c>
+    </row>
+    <row r="20" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E20">
+        <f t="shared" si="2"/>
+        <v>0.54999999999999993</v>
+      </c>
+      <c r="F20">
+        <f t="shared" si="1"/>
+        <v>67.857000000000014</v>
+      </c>
+    </row>
+    <row r="21" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E21">
+        <f t="shared" si="2"/>
+        <v>0.6</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="1"/>
+        <v>60.713999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E22">
+        <f t="shared" si="2"/>
+        <v>0.65</v>
+      </c>
+      <c r="F22">
+        <f t="shared" si="1"/>
+        <v>53.570999999999998</v>
+      </c>
+    </row>
+    <row r="23" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E23">
+        <f t="shared" si="2"/>
+        <v>0.70000000000000007</v>
+      </c>
+      <c r="F23">
+        <f t="shared" si="1"/>
+        <v>46.427999999999983</v>
+      </c>
+      <c r="H23">
+        <v>0.7</v>
+      </c>
+      <c r="I23">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E24">
+        <f t="shared" si="2"/>
+        <v>0.75000000000000011</v>
+      </c>
+      <c r="F24">
+        <f t="shared" si="1"/>
+        <v>39.284999999999982</v>
+      </c>
+    </row>
+    <row r="25" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E25">
+        <f t="shared" si="2"/>
+        <v>0.80000000000000016</v>
+      </c>
+      <c r="F25">
+        <f t="shared" si="1"/>
+        <v>32.141999999999967</v>
+      </c>
+    </row>
+    <row r="26" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E26">
+        <f t="shared" si="2"/>
+        <v>0.8500000000000002</v>
+      </c>
+      <c r="F26">
+        <f t="shared" si="1"/>
+        <v>24.998999999999967</v>
+      </c>
+    </row>
+    <row r="27" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E27">
+        <f t="shared" si="2"/>
+        <v>0.90000000000000024</v>
+      </c>
+      <c r="F27">
+        <f t="shared" si="1"/>
+        <v>17.855999999999966</v>
+      </c>
+    </row>
+    <row r="28" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E28">
+        <f t="shared" si="2"/>
+        <v>0.95000000000000029</v>
+      </c>
+      <c r="F28">
+        <f t="shared" si="1"/>
+        <v>10.712999999999965</v>
+      </c>
+      <c r="H28">
+        <v>0.94</v>
+      </c>
+      <c r="I28">
+        <v>26</v>
+      </c>
+      <c r="J28">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="29" spans="5:10" x14ac:dyDescent="0.35">
+      <c r="E29">
+        <f t="shared" si="2"/>
+        <v>1.0000000000000002</v>
+      </c>
+      <c r="F29">
+        <f t="shared" si="1"/>
+        <v>3.5699999999999648</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>

</xml_diff>